<commit_message>
update the readme.md file
</commit_message>
<xml_diff>
--- a/documents/Product Labeling Status.xlsx
+++ b/documents/Product Labeling Status.xlsx
@@ -5,21 +5,22 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\document\unlon object detect\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\unknown_product_detection\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14380" windowHeight="4190" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="26">
   <si>
     <t>S.No.</t>
   </si>
@@ -103,7 +104,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -123,8 +124,24 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -143,8 +160,14 @@
         <bgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -235,6 +258,133 @@
       <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -242,7 +392,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -267,6 +417,18 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -499,7 +661,7 @@
     <col min="5" max="5" width="17.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -772,4 +934,95 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5.81640625" customWidth="1"/>
+    <col min="2" max="2" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="14" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="25" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="20">
+        <v>1</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="21">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="15">
+        <v>2</v>
+      </c>
+      <c r="B3" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="16">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="15">
+        <v>3</v>
+      </c>
+      <c r="B4" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="16">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="15">
+        <v>4</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="16">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="17">
+        <v>5</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="18">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="17"/>
+      <c r="B7" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="18">
+        <v>1878</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>